<commit_message>
chore: populate live alert data — 26 alerts, 2 insider buys, 50 contracts
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -152,8 +152,6 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -596,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -621,7 +619,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-05 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-06 04:16 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +639,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.911</v>
+        <v>0.926</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -657,7 +655,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -673,7 +671,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>346.54</v>
+        <v>346.32</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>178.1</v>
+        <v>178.25</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +701,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.946</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -734,79 +732,64 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>comps_percentile</t>
+          <t>dcf_margin</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.889</v>
+        <v>1</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Peer-relative ranking of P/E, EV/EBITDA, EV/Rev</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>dcf_margin</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
           <t>Normalized (intrinsic − market) / market, clipped ±50%</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Honest caveats (read before acting)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Honest caveats (read before acting)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
+          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
+          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
+          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
+          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>This is a SIGNAL screen, not an investment thesis. Verify with primary filings before acting.</t>
         </is>
@@ -816,7 +799,6 @@
   <mergeCells count="11">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
@@ -825,6 +807,7 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -891,7 +874,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04532000064849853</v>
+        <v>0.0453600025177002</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1203,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>615435154.1830432</v>
+        <v>615435156.2861151</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1224,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>178.1</v>
+        <v>178.25</v>
       </c>
     </row>
     <row r="38">
@@ -1446,7 +1429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1520,266 +1503,68 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>109609000960</v>
+        <v>109701316608</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.6</v>
+        <v>14.62</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.66</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.53</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ADBE</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Adobe Inc.</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="n">
-        <v>101842231296</v>
-      </c>
-      <c r="D6" s="34" t="n">
-        <v>14.682984</v>
-      </c>
-      <c r="E6" s="34" t="n">
-        <v>10.953</v>
-      </c>
-      <c r="F6" s="34" t="n">
-        <v>4.262</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AMAT</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Applied Materials, Inc.</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="n">
-        <v>371868762112</v>
-      </c>
-      <c r="D7" s="34" t="n">
-        <v>44.01997</v>
-      </c>
-      <c r="E7" s="34" t="n">
-        <v>42.842</v>
-      </c>
-      <c r="F7" s="34" t="n">
-        <v>13.691</v>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Peer median</t>
+        </is>
+      </c>
+      <c r="D7" s="33">
+        <f>MEDIAN(D6:D5)</f>
+        <v/>
+      </c>
+      <c r="E7" s="33">
+        <f>MEDIAN(E6:E5)</f>
+        <v/>
+      </c>
+      <c r="F7" s="33">
+        <f>MEDIAN(F6:F5)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>APH</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Amphenol Corporation</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="n">
-        <v>173204701184</v>
-      </c>
-      <c r="D8" s="34" t="n">
-        <v>40.456894</v>
-      </c>
-      <c r="E8" s="34" t="n">
-        <v>23.845</v>
-      </c>
-      <c r="F8" s="34" t="n">
-        <v>7.522</v>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Peer mean</t>
+        </is>
+      </c>
+      <c r="D8" s="33">
+        <f>AVERAGE(D6:D5)</f>
+        <v/>
+      </c>
+      <c r="E8" s="33">
+        <f>AVERAGE(E6:E5)</f>
+        <v/>
+      </c>
+      <c r="F8" s="33">
+        <f>AVERAGE(F6:F5)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>INFY</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Infosys Limited</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="n">
-        <v>50384887808</v>
-      </c>
-      <c r="D9" s="34" t="n">
-        <v>15.55625</v>
-      </c>
-      <c r="E9" s="34" t="n">
-        <v>10.882</v>
-      </c>
-      <c r="F9" s="34" t="n">
-        <v>2.39</v>
-      </c>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Target percentile vs peers</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="n"/>
+      <c r="E9" s="34" t="n"/>
+      <c r="F9" s="34" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>KLAC</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>KLA Corporation</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="n">
-        <v>259814866944</v>
-      </c>
-      <c r="D10" s="34" t="n">
-        <v>56.217495</v>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>47.788</v>
-      </c>
-      <c r="F10" s="34" t="n">
-        <v>21.346</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LDOS</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Leidos Holdings, Inc.</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="n">
-        <v>15766579200</v>
-      </c>
-      <c r="D11" s="34" t="n">
-        <v>11.47848</v>
-      </c>
-      <c r="E11" s="34" t="n">
-        <v>9.238</v>
-      </c>
-      <c r="F11" s="34" t="n">
-        <v>1.281</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Palo Alto Networks, Inc.</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="n">
-        <v>224410255360</v>
-      </c>
-      <c r="D12" s="34" t="n">
-        <v>241.5351</v>
-      </c>
-      <c r="E12" s="34" t="n">
-        <v>152.752</v>
-      </c>
-      <c r="F12" s="34" t="n">
-        <v>21.365</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>QCOM</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>QUALCOMM Incorporated</t>
-        </is>
-      </c>
-      <c r="C13" s="33" t="n">
-        <v>231816757248</v>
-      </c>
-      <c r="D13" s="34" t="n">
-        <v>23.67492</v>
-      </c>
-      <c r="E13" s="34" t="n">
-        <v>20.089</v>
-      </c>
-      <c r="F13" s="34" t="n">
-        <v>5.87</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Peer median</t>
-        </is>
-      </c>
-      <c r="D15" s="35">
-        <f>MEDIAN(D6:D13)</f>
-        <v/>
-      </c>
-      <c r="E15" s="35">
-        <f>MEDIAN(E6:E13)</f>
-        <v/>
-      </c>
-      <c r="F15" s="35">
-        <f>MEDIAN(F6:F13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Peer mean</t>
-        </is>
-      </c>
-      <c r="D16" s="35">
-        <f>AVERAGE(D6:D13)</f>
-        <v/>
-      </c>
-      <c r="E16" s="35">
-        <f>AVERAGE(E6:E13)</f>
-        <v/>
-      </c>
-      <c r="F16" s="35">
-        <f>AVERAGE(F6:F13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Target percentile vs peers</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="E17" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="36" t="n">
-        <v>0.167</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>(higher pct = more expensive than peers)</t>
         </is>

</xml_diff>

<commit_message>
n8n board refresh 2026-06-06T17:39:10Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -152,6 +152,8 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -594,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -619,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-06 04:16 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-06 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -639,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.926</v>
+        <v>0.911</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -655,7 +657,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -732,64 +734,79 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>comps_percentile</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Peer-relative ranking of P/E, EV/EBITDA, EV/Rev</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>dcf_margin</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Normalized (intrinsic − market) / market, clipped ±50%</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Honest caveats (read before acting)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
-        </is>
-      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
+          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
+          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
+          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
+          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>This is a SIGNAL screen, not an investment thesis. Verify with primary filings before acting.</t>
         </is>
@@ -799,6 +816,7 @@
   <mergeCells count="11">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
@@ -807,7 +825,6 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -874,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.0453600025177002</v>
+        <v>0.04535999774932861</v>
       </c>
     </row>
     <row r="6">
@@ -1429,7 +1446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1515,56 +1532,254 @@
         <v>1.52</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Adobe Inc.</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="n">
+        <v>101632049152</v>
+      </c>
+      <c r="D6" s="34" t="n">
+        <v>14.661225</v>
+      </c>
+      <c r="E6" s="34" t="n">
+        <v>10.656</v>
+      </c>
+      <c r="F6" s="34" t="n">
+        <v>4.147</v>
+      </c>
+    </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Applied Materials, Inc.</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="n">
+        <v>359671562240</v>
+      </c>
+      <c r="D7" s="34" t="n">
+        <v>42.53615</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>38.674</v>
+      </c>
+      <c r="F7" s="34" t="n">
+        <v>12.359</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>APH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Amphenol Corporation</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>170768842752</v>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>39.88793</v>
+      </c>
+      <c r="E8" s="34" t="n">
+        <v>22.646</v>
+      </c>
+      <c r="F8" s="34" t="n">
+        <v>7.144</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>50202697728</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>15.499999</v>
+      </c>
+      <c r="E9" s="34" t="n">
+        <v>10.727</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>2.356</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KLA Corporation</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="n">
+        <v>252006612992</v>
+      </c>
+      <c r="D10" s="34" t="n">
+        <v>54.651558</v>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>43.279</v>
+      </c>
+      <c r="F10" s="34" t="n">
+        <v>19.333</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LDOS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Leidos Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>15651485696</v>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>11.394689</v>
+      </c>
+      <c r="E11" s="34" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="F11" s="34" t="n">
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Palo Alto Networks, Inc.</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="n">
+        <v>221720739840</v>
+      </c>
+      <c r="D12" s="34" t="n">
+        <v>238.64035</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>148.797</v>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>20.812</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>QUALCOMM Incorporated</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="n">
+        <v>227600760832</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>23.194414</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>5.239</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Peer median</t>
         </is>
       </c>
-      <c r="D7" s="33">
-        <f>MEDIAN(D6:D5)</f>
-        <v/>
-      </c>
-      <c r="E7" s="33">
-        <f>MEDIAN(E6:E5)</f>
-        <v/>
-      </c>
-      <c r="F7" s="33">
-        <f>MEDIAN(F6:F5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="D15" s="35">
+        <f>MEDIAN(D6:D13)</f>
+        <v/>
+      </c>
+      <c r="E15" s="35">
+        <f>MEDIAN(E6:E13)</f>
+        <v/>
+      </c>
+      <c r="F15" s="35">
+        <f>MEDIAN(F6:F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Peer mean</t>
         </is>
       </c>
-      <c r="D8" s="33">
-        <f>AVERAGE(D6:D5)</f>
-        <v/>
-      </c>
-      <c r="E8" s="33">
-        <f>AVERAGE(E6:E5)</f>
-        <v/>
-      </c>
-      <c r="F8" s="33">
-        <f>AVERAGE(F6:F5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="D16" s="35">
+        <f>AVERAGE(D6:D13)</f>
+        <v/>
+      </c>
+      <c r="E16" s="35">
+        <f>AVERAGE(E6:E13)</f>
+        <v/>
+      </c>
+      <c r="F16" s="35">
+        <f>AVERAGE(F6:F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Target percentile vs peers</t>
         </is>
       </c>
-      <c r="D9" s="34" t="n"/>
-      <c r="E9" s="34" t="n"/>
-      <c r="F9" s="34" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="D17" s="36" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="E17" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="36" t="n">
+        <v>0.167</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>(higher pct = more expensive than peers)</t>
         </is>

</xml_diff>

<commit_message>
n8n board refresh 2026-06-15T17:48:22Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-06 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-15 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.911</v>
+        <v>0.893</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>346.32</v>
+        <v>350.01</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>178.25</v>
+        <v>168.41</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.9429999999999999</v>
+        <v>1.078</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.777</v>
+        <v>0.798</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.889</v>
+        <v>0.833</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04535999774932861</v>
+        <v>0.04468999862670898</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>615435156.2861151</v>
+        <v>615435127.1302179</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>178.25</v>
+        <v>168.41</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>109701316608</v>
+        <v>103645429760</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.62</v>
+        <v>13.82</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.630000000000001</v>
+        <v>8.25</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.52</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>101632049152</v>
+        <v>84111998976</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>14.661225</v>
+        <v>11.904749</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.656</v>
+        <v>8.723000000000001</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>4.147</v>
+        <v>3.312</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>359671562240</v>
+        <v>469361000448</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>42.53615</v>
+        <v>55.71772</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>38.674</v>
+        <v>48.453</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>12.359</v>
+        <v>15.484</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>170768842752</v>
+        <v>195151970304</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>39.88793</v>
+        <v>45.583305</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>22.646</v>
+        <v>24.903</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.144</v>
+        <v>7.856</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>50202697728</v>
+        <v>47773540352</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>15.499999</v>
+        <v>14.75</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>10.727</v>
+        <v>20.853</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>2.356</v>
+        <v>4.581</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>252006612992</v>
+        <v>330912169984</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>54.651558</v>
+        <v>71.56074</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>43.279</v>
+        <v>57.038</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>19.333</v>
+        <v>25.479</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>15651485696</v>
+        <v>14543944704</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>11.394689</v>
+        <v>10.578682</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.23</v>
+        <v>9.111000000000001</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.28</v>
+        <v>1.264</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>221720739840</v>
+        <v>231032127488</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>238.64035</v>
+        <v>246.50002</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>148.797</v>
+        <v>152.955</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>20.812</v>
+        <v>21.393</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>227600760832</v>
+        <v>233827270656</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>23.194414</v>
+        <v>23.880249</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>17.93</v>
+        <v>17.588</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>5.239</v>
+        <v>5.139</v>
       </c>
     </row>
     <row r="15">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D17" s="36" t="n">
-        <v>0.167</v>
+        <v>0.333</v>
       </c>
       <c r="E17" s="36" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-06-16T17:47:05Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-15 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-16 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.893</v>
+        <v>0.894</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>350.01</v>
+        <v>352.42</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>168.41</v>
+        <v>165.975</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.078</v>
+        <v>1.123</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.798</v>
+        <v>0.803</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04468999862670898</v>
+        <v>0.04425999641418457</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>615435127.1302179</v>
+        <v>615435160.8133755</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>168.41</v>
+        <v>165.975</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>103645429760</v>
+        <v>102146850816</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.82</v>
+        <v>13.6</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.25</v>
+        <v>8.01</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.46</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>84111998976</v>
+        <v>82250702848</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>11.904749</v>
+        <v>11.837529</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>8.723000000000001</v>
+        <v>8.58</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.312</v>
+        <v>3.313</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>469361000448</v>
+        <v>459142758400</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>55.71772</v>
+        <v>54.55613</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>48.453</v>
+        <v>50.039</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>15.484</v>
+        <v>15.991</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>195151970304</v>
+        <v>195816423424</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>45.583305</v>
+        <v>45.870316</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.903</v>
+        <v>25.624</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.856</v>
+        <v>8.083</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>47773540352</v>
+        <v>48704716800</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.75</v>
+        <v>15.037499</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>20.853</v>
+        <v>20.597</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.581</v>
+        <v>4.524</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>330912169984</v>
+        <v>316190425088</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>71.56074</v>
+        <v>68.37712000000001</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>57.038</v>
+        <v>57.458</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>25.479</v>
+        <v>25.666</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14543944704</v>
+        <v>14396145664</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>10.578682</v>
+        <v>10.47118</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.111000000000001</v>
+        <v>8.715999999999999</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.264</v>
+        <v>1.209</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>231032127488</v>
+        <v>227140517888</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>246.50002</v>
+        <v>244.4737</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>152.955</v>
+        <v>155.658</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>21.393</v>
+        <v>21.771</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>233827270656</v>
+        <v>230267387904</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>23.880249</v>
+        <v>23.491398</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>17.588</v>
+        <v>18.325</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>5.139</v>
+        <v>5.355</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-17T17:46:43Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-16 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-17 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.894</v>
+        <v>0.896</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>352.42</v>
+        <v>352.08</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>165.975</v>
+        <v>160.895</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.123</v>
+        <v>1.188</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.803</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04425999641418457</v>
+        <v>0.04432000160217285</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>615435160.8133755</v>
+        <v>615435156.7916964</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>165.975</v>
+        <v>160.895</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>102146850816</v>
+        <v>99020439552</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.6</v>
+        <v>13.19</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.01</v>
+        <v>8.02</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>1.42</v>
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>82250702848</v>
+        <v>80390406144</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>11.837529</v>
+        <v>11.569795</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>8.58</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.313</v>
+        <v>3.328</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>459142758400</v>
+        <v>484418453504</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>54.55613</v>
+        <v>57.396988</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>50.039</v>
+        <v>48.537</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>15.991</v>
+        <v>15.511</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>195816423424</v>
+        <v>200663547904</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>45.870316</v>
+        <v>46.87069</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>25.624</v>
+        <v>25.657</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>8.083</v>
+        <v>8.093999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>48704716800</v>
+        <v>48239128576</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>15.037499</v>
+        <v>14.89375</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>20.597</v>
+        <v>21.273</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.524</v>
+        <v>4.673</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>316190425088</v>
+        <v>316340666368</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>68.37712000000001</v>
+        <v>68.40961</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>57.458</v>
+        <v>53.196</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>25.666</v>
+        <v>23.762</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14396145664</v>
+        <v>13900552192</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>10.47118</v>
+        <v>10.110704</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.715999999999999</v>
+        <v>8.663</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.209</v>
+        <v>1.202</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>227140517888</v>
+        <v>230681690112</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>244.4737</v>
+        <v>246.1261</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>155.658</v>
+        <v>153.109</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>21.771</v>
+        <v>21.415</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>230267387904</v>
+        <v>229582290944</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>23.491398</v>
+        <v>23.446718</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>18.325</v>
+        <v>17.778</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>5.355</v>
+        <v>5.195</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-18T17:47:43Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -20,11 +20,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="169" formatCode="+0.0%;-0.0%"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -126,22 +126,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,9 +149,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -596,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -621,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-17 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-18 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.896</v>
+        <v>0.888</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -657,7 +656,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -672,8 +671,10 @@
           <t>DCF intrinsic value / share</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>352.08</v>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>160.895</v>
+        <v>128.16</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -702,8 +703,10 @@
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>1.188</v>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -726,8 +729,8 @@
           <t>value_score</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
-        <v>0.8139999999999999</v>
+      <c r="B13" s="8" t="n">
+        <v>0.886</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -737,8 +740,8 @@
           <t>comps_percentile</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
-        <v>0.833</v>
+      <c r="B14" s="8" t="n">
+        <v>0.889</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -746,67 +749,52 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>dcf_margin</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Normalized (intrinsic − market) / market, clipped ±50%</t>
-        </is>
-      </c>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Honest caveats (read before acting)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Honest caveats (read before acting)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
+          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
+          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
+          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
+          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>This is a SIGNAL screen, not an investment thesis. Verify with primary filings before acting.</t>
         </is>
@@ -816,7 +804,6 @@
   <mergeCells count="11">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
@@ -825,6 +812,7 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -890,8 +878,8 @@
           <t>Risk-free rate (10y Treasury)</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
-        <v>0.04432000160217285</v>
+      <c r="B5" s="9" t="n">
+        <v>0.04438000202178955</v>
       </c>
     </row>
     <row r="6">
@@ -900,7 +888,7 @@
           <t>Equity risk premium (ERP)</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -910,7 +898,7 @@
           <t>Beta (levered)</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <v>1.069</v>
       </c>
     </row>
@@ -920,7 +908,7 @@
           <t>Credit spread over risk-free</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="9" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -930,7 +918,7 @@
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="9" t="n">
         <v>0.21</v>
       </c>
     </row>
@@ -940,7 +928,7 @@
           <t>Equity weight (cap structure)</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="11" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -950,7 +938,7 @@
           <t>FCF growth (flat, faded avg)</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="9" t="n">
         <v>0.05241951788891955</v>
       </c>
     </row>
@@ -960,7 +948,7 @@
           <t>Terminal growth rate</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="9" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -970,7 +958,7 @@
           <t>Latest FCF ($, base year)</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="12" t="n">
         <v>10874360000</v>
       </c>
     </row>
@@ -980,7 +968,7 @@
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="13">
         <f>B5+B7*B6</f>
         <v/>
       </c>
@@ -991,18 +979,18 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="13">
         <f>(B5+B8)*(1-B9)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <f>B10*B15+(1-B10)*B16</f>
         <v/>
       </c>
@@ -1049,23 +1037,23 @@
           <t>Projected FCF</t>
         </is>
       </c>
-      <c r="B22" s="17">
+      <c r="B22" s="16">
         <f>$B$13*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="16">
         <f>B22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="16">
         <f>C22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="16">
         <f>D22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="F22" s="17">
+      <c r="F22" s="16">
         <f>E22*(1+$B$11)</f>
         <v/>
       </c>
@@ -1076,23 +1064,23 @@
           <t>Discount factor</t>
         </is>
       </c>
-      <c r="B23" s="18">
+      <c r="B23" s="17">
         <f>1/(1+$B$17)^1</f>
         <v/>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="17">
         <f>1/(1+$B$17)^2</f>
         <v/>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="17">
         <f>1/(1+$B$17)^3</f>
         <v/>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="17">
         <f>1/(1+$B$17)^4</f>
         <v/>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="17">
         <f>1/(1+$B$17)^5</f>
         <v/>
       </c>
@@ -1103,23 +1091,23 @@
           <t>PV of FCF</t>
         </is>
       </c>
-      <c r="B24" s="17">
+      <c r="B24" s="16">
         <f>B22*B23</f>
         <v/>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="16">
         <f>C22*C23</f>
         <v/>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="16">
         <f>D22*D23</f>
         <v/>
       </c>
-      <c r="E24" s="17">
+      <c r="E24" s="16">
         <f>E22*E23</f>
         <v/>
       </c>
-      <c r="F24" s="17">
+      <c r="F24" s="16">
         <f>F22*F23</f>
         <v/>
       </c>
@@ -1130,7 +1118,7 @@
           <t>Sum of PV (explicit 5y)</t>
         </is>
       </c>
-      <c r="B26" s="17">
+      <c r="B26" s="16">
         <f>SUM(B24:F24)</f>
         <v/>
       </c>
@@ -1141,7 +1129,7 @@
           <t>Terminal value (Gordon)</t>
         </is>
       </c>
-      <c r="B27" s="17">
+      <c r="B27" s="16">
         <f>F22*(1+B12)/(B17-B12)</f>
         <v/>
       </c>
@@ -1152,18 +1140,18 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="B28" s="17">
+      <c r="B28" s="16">
         <f>B27/(1+B17)^5</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B29" s="20">
+      <c r="B29" s="19">
         <f>B26+B28</f>
         <v/>
       </c>
@@ -1188,7 +1176,7 @@
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n">
+      <c r="B32" s="12" t="n">
         <v>8347366912</v>
       </c>
     </row>
@@ -1198,7 +1186,7 @@
           <t>Plus: cash &amp; ST investments</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="12" t="n">
         <v>9405595648</v>
       </c>
     </row>
@@ -1208,7 +1196,7 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="B34" s="17">
+      <c r="B34" s="16">
         <f>B29-B32+B33</f>
         <v/>
       </c>
@@ -1219,17 +1207,17 @@
           <t>Diluted shares outstanding</t>
         </is>
       </c>
-      <c r="B35" s="21" t="n">
-        <v>615435156.7916964</v>
+      <c r="B35" s="20" t="n">
+        <v>615435122.0973783</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Intrinsic per share</t>
         </is>
       </c>
-      <c r="B36" s="22">
+      <c r="B36" s="21">
         <f>B34/B35</f>
         <v/>
       </c>
@@ -1240,17 +1228,17 @@
           <t>Current market price</t>
         </is>
       </c>
-      <c r="B37" s="23" t="n">
-        <v>160.895</v>
+      <c r="B37" s="22" t="n">
+        <v>128.16</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B38" s="24">
+      <c r="B38" s="23">
         <f>(B36-B37)/B37</f>
         <v/>
       </c>
@@ -1270,158 +1258,158 @@
       <c r="H41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="inlineStr">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>WACC ↓ / TermG →</t>
         </is>
       </c>
-      <c r="B42" s="26">
+      <c r="B42" s="25">
         <f>$B$12+-0.01</f>
         <v/>
       </c>
-      <c r="C42" s="26">
+      <c r="C42" s="25">
         <f>$B$12+-0.005</f>
         <v/>
       </c>
-      <c r="D42" s="26">
+      <c r="D42" s="25">
         <f>$B$12+0.0</f>
         <v/>
       </c>
-      <c r="E42" s="26">
+      <c r="E42" s="25">
         <f>$B$12+0.005</f>
         <v/>
       </c>
-      <c r="F42" s="26">
+      <c r="F42" s="25">
         <f>$B$12+0.01</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="26">
+      <c r="A43" s="25">
         <f>$B$17+-0.01</f>
         <v/>
       </c>
-      <c r="B43" s="27">
+      <c r="B43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A43-B$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C43" s="27">
+      <c r="C43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A43-C$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D43" s="27">
+      <c r="D43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A43-D$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E43" s="27">
+      <c r="E43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A43-E$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F43" s="27">
+      <c r="F43" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A43-F$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="26">
+      <c r="A44" s="25">
         <f>$B$17+-0.005</f>
         <v/>
       </c>
-      <c r="B44" s="27">
+      <c r="B44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A44-B$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C44" s="27">
+      <c r="C44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A44-C$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D44" s="27">
+      <c r="D44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A44-D$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E44" s="27">
+      <c r="E44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A44-E$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F44" s="27">
+      <c r="F44" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A44-F$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="26">
+      <c r="A45" s="25">
         <f>$B$17+0.0</f>
         <v/>
       </c>
-      <c r="B45" s="27">
+      <c r="B45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A45-B$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C45" s="27">
+      <c r="C45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A45-C$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D45" s="28">
+      <c r="D45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A45-D$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E45" s="27">
+      <c r="E45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A45-E$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F45" s="27">
+      <c r="F45" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A45-F$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="26">
+      <c r="A46" s="25">
         <f>$B$17+0.005</f>
         <v/>
       </c>
-      <c r="B46" s="27">
+      <c r="B46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A46-B$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C46" s="27">
+      <c r="C46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A46-C$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D46" s="27">
+      <c r="D46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A46-D$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E46" s="27">
+      <c r="E46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A46-E$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F46" s="27">
+      <c r="F46" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A46-F$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="26">
+      <c r="A47" s="25">
         <f>$B$17+0.01</f>
         <v/>
       </c>
-      <c r="B47" s="27">
+      <c r="B47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A47-B$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C47" s="27">
+      <c r="C47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A47-C$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D47" s="27">
+      <c r="D47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A47-D$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E47" s="27">
+      <c r="E47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A47-E$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F47" s="27">
+      <c r="F47" s="26">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A47-F$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
@@ -1477,58 +1465,58 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>P/E (TTM)</t>
         </is>
       </c>
-      <c r="E4" s="29" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="F4" s="29" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>EV/Revenue</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>ACN</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Accenture plc</t>
         </is>
       </c>
-      <c r="C5" s="31" t="n">
-        <v>99020439552</v>
-      </c>
-      <c r="D5" s="32" t="n">
-        <v>13.19</v>
-      </c>
-      <c r="E5" s="32" t="n">
+      <c r="C5" s="30" t="n">
+        <v>78874165248</v>
+      </c>
+      <c r="D5" s="31" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E5" s="31" t="n">
         <v>8.02</v>
       </c>
-      <c r="F5" s="32" t="n">
+      <c r="F5" s="31" t="n">
         <v>1.42</v>
       </c>
     </row>
@@ -1543,16 +1531,16 @@
           <t>Adobe Inc.</t>
         </is>
       </c>
-      <c r="C6" s="33" t="n">
-        <v>80390406144</v>
-      </c>
-      <c r="D6" s="34" t="n">
-        <v>11.569795</v>
-      </c>
-      <c r="E6" s="34" t="n">
+      <c r="C6" s="32" t="n">
+        <v>77538852864</v>
+      </c>
+      <c r="D6" s="33" t="n">
+        <v>11.1594</v>
+      </c>
+      <c r="E6" s="33" t="n">
         <v>8.619999999999999</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="33" t="n">
         <v>3.328</v>
       </c>
     </row>
@@ -1567,16 +1555,16 @@
           <t>Applied Materials, Inc.</t>
         </is>
       </c>
-      <c r="C7" s="33" t="n">
-        <v>484418453504</v>
-      </c>
-      <c r="D7" s="34" t="n">
-        <v>57.396988</v>
-      </c>
-      <c r="E7" s="34" t="n">
+      <c r="C7" s="32" t="n">
+        <v>490285826048</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>58.092194</v>
+      </c>
+      <c r="E7" s="33" t="n">
         <v>48.537</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="33" t="n">
         <v>15.511</v>
       </c>
     </row>
@@ -1591,16 +1579,16 @@
           <t>Amphenol Corporation</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
-        <v>200663547904</v>
-      </c>
-      <c r="D8" s="34" t="n">
-        <v>46.87069</v>
-      </c>
-      <c r="E8" s="34" t="n">
+      <c r="C8" s="32" t="n">
+        <v>203382374400</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <v>47.50575</v>
+      </c>
+      <c r="E8" s="33" t="n">
         <v>25.657</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="33" t="n">
         <v>8.093999999999999</v>
       </c>
     </row>
@@ -1615,16 +1603,16 @@
           <t>Infosys Limited</t>
         </is>
       </c>
-      <c r="C9" s="33" t="n">
-        <v>48239128576</v>
-      </c>
-      <c r="D9" s="34" t="n">
-        <v>14.89375</v>
-      </c>
-      <c r="E9" s="34" t="n">
+      <c r="C9" s="32" t="n">
+        <v>43421290496</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>13.40625</v>
+      </c>
+      <c r="E9" s="33" t="n">
         <v>21.273</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="33" t="n">
         <v>4.673</v>
       </c>
     </row>
@@ -1639,16 +1627,16 @@
           <t>KLA Corporation</t>
         </is>
       </c>
-      <c r="C10" s="33" t="n">
-        <v>316340666368</v>
-      </c>
-      <c r="D10" s="34" t="n">
-        <v>68.40961</v>
-      </c>
-      <c r="E10" s="34" t="n">
+      <c r="C10" s="32" t="n">
+        <v>339226624000</v>
+      </c>
+      <c r="D10" s="33" t="n">
+        <v>73.35876</v>
+      </c>
+      <c r="E10" s="33" t="n">
         <v>53.196</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="33" t="n">
         <v>23.762</v>
       </c>
     </row>
@@ -1663,16 +1651,16 @@
           <t>Leidos Holdings, Inc.</t>
         </is>
       </c>
-      <c r="C11" s="33" t="n">
-        <v>13900552192</v>
-      </c>
-      <c r="D11" s="34" t="n">
-        <v>10.110704</v>
-      </c>
-      <c r="E11" s="34" t="n">
+      <c r="C11" s="32" t="n">
+        <v>13465962496</v>
+      </c>
+      <c r="D11" s="33" t="n">
+        <v>9.794601</v>
+      </c>
+      <c r="E11" s="33" t="n">
         <v>8.663</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="33" t="n">
         <v>1.202</v>
       </c>
     </row>
@@ -1687,16 +1675,16 @@
           <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
-      <c r="C12" s="33" t="n">
-        <v>230681690112</v>
-      </c>
-      <c r="D12" s="34" t="n">
-        <v>246.1261</v>
-      </c>
-      <c r="E12" s="34" t="n">
+      <c r="C12" s="32" t="n">
+        <v>232666038272</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <v>248.2433</v>
+      </c>
+      <c r="E12" s="33" t="n">
         <v>153.109</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="33" t="n">
         <v>21.415</v>
       </c>
     </row>
@@ -1711,16 +1699,16 @@
           <t>QUALCOMM Incorporated</t>
         </is>
       </c>
-      <c r="C13" s="33" t="n">
-        <v>229582290944</v>
-      </c>
-      <c r="D13" s="34" t="n">
-        <v>23.446718</v>
-      </c>
-      <c r="E13" s="34" t="n">
+      <c r="C13" s="32" t="n">
+        <v>238657208320</v>
+      </c>
+      <c r="D13" s="33" t="n">
+        <v>24.37352</v>
+      </c>
+      <c r="E13" s="33" t="n">
         <v>17.778</v>
       </c>
-      <c r="F13" s="34" t="n">
+      <c r="F13" s="33" t="n">
         <v>5.195</v>
       </c>
     </row>
@@ -1730,15 +1718,15 @@
           <t>Peer median</t>
         </is>
       </c>
-      <c r="D15" s="35">
+      <c r="D15" s="34">
         <f>MEDIAN(D6:D13)</f>
         <v/>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="34">
         <f>MEDIAN(E6:E13)</f>
         <v/>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="34">
         <f>MEDIAN(F6:F13)</f>
         <v/>
       </c>
@@ -1749,15 +1737,15 @@
           <t>Peer mean</t>
         </is>
       </c>
-      <c r="D16" s="35">
+      <c r="D16" s="34">
         <f>AVERAGE(D6:D13)</f>
         <v/>
       </c>
-      <c r="E16" s="35">
+      <c r="E16" s="34">
         <f>AVERAGE(E6:E13)</f>
         <v/>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="34">
         <f>AVERAGE(F6:F13)</f>
         <v/>
       </c>
@@ -1768,13 +1756,13 @@
           <t>Target percentile vs peers</t>
         </is>
       </c>
-      <c r="D17" s="36" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="E17" s="36" t="n">
+      <c r="D17" s="35" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="E17" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="36" t="n">
+      <c r="F17" s="35" t="n">
         <v>0.167</v>
       </c>
     </row>

</xml_diff>

<commit_message>
n8n board refresh 2026-06-19T17:46:42Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-18 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-19 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>128.16</v>
+        <v>127.98</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.886</v>
+        <v>0.887</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04438000202178955</v>
+        <v>0.044509997</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>615435122.0973783</v>
+        <v>615435169.7452726</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>128.16</v>
+        <v>127.98</v>
       </c>
     </row>
     <row r="38">
@@ -1508,10 +1508,10 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>78874165248</v>
+        <v>78763393024</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>10.5</v>
+        <v>10.49</v>
       </c>
       <c r="E5" s="31" t="n">
         <v>8.02</v>
@@ -1532,10 +1532,10 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>77538852864</v>
+        <v>77576101888</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>11.1594</v>
+        <v>11.164761</v>
       </c>
       <c r="E6" s="33" t="n">
         <v>8.619999999999999</v>
@@ -1556,10 +1556,10 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>490285826048</v>
+        <v>489960275968</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>58.092194</v>
+        <v>58.05362</v>
       </c>
       <c r="E7" s="33" t="n">
         <v>48.537</v>
@@ -1580,10 +1580,10 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>203382374400</v>
+        <v>201709256704</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>47.50575</v>
+        <v>47.114944</v>
       </c>
       <c r="E8" s="33" t="n">
         <v>25.657</v>
@@ -1604,10 +1604,10 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>43421290496</v>
+        <v>42793754624</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>13.40625</v>
+        <v>13.2125</v>
       </c>
       <c r="E9" s="33" t="n">
         <v>21.273</v>
@@ -1628,10 +1628,10 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>339226624000</v>
+        <v>339056787456</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>73.35876</v>
+        <v>73.32204</v>
       </c>
       <c r="E10" s="33" t="n">
         <v>53.196</v>
@@ -1652,10 +1652,10 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>13465962496</v>
+        <v>13474139136</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>9.794601</v>
+        <v>9.800549</v>
       </c>
       <c r="E11" s="33" t="n">
         <v>8.663</v>
@@ -1676,10 +1676,10 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>232666038272</v>
+        <v>234540695552</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>248.2433</v>
+        <v>250.24348</v>
       </c>
       <c r="E12" s="33" t="n">
         <v>153.109</v>
@@ -1700,10 +1700,10 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>238657208320</v>
+        <v>238319943680</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>24.37352</v>
+        <v>24.339075</v>
       </c>
       <c r="E13" s="33" t="n">
         <v>17.778</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-02T17:39:49Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-19 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-02 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.888</v>
+        <v>0.92</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>127.98</v>
+        <v>137.645</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.887</v>
+        <v>0.873</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>0.889</v>
+        <v>0.944</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.044509997</v>
+        <v>0.04480999946594239</v>
       </c>
     </row>
     <row r="6">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>8347366912</v>
+        <v>8388769792</v>
       </c>
     </row>
     <row r="33">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="B33" s="12" t="n">
-        <v>9405595648</v>
+        <v>10171567104</v>
       </c>
     </row>
     <row r="34">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>615435169.7452726</v>
+        <v>611942072.6651894</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>127.98</v>
+        <v>137.645</v>
       </c>
     </row>
     <row r="38">
@@ -1508,16 +1508,16 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>78763393024</v>
+        <v>84230766592</v>
       </c>
       <c r="D5" s="31" t="n">
-        <v>10.49</v>
+        <v>10.99</v>
       </c>
       <c r="E5" s="31" t="n">
-        <v>8.02</v>
+        <v>6.19</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>1.42</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="6">
@@ -1532,16 +1532,16 @@
         </is>
       </c>
       <c r="C6" s="32" t="n">
-        <v>77576101888</v>
+        <v>87986429952</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>11.164761</v>
+        <v>12.655775</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>8.619999999999999</v>
+        <v>8.769</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>3.328</v>
+        <v>3.386</v>
       </c>
     </row>
     <row r="7">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>489960275968</v>
+        <v>465839783936</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>58.05362</v>
+        <v>55.299717</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>48.537</v>
+        <v>55.614</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>15.511</v>
+        <v>17.772</v>
       </c>
     </row>
     <row r="8">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>201709256704</v>
+        <v>199986921472</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>47.114944</v>
+        <v>46.712643</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>25.657</v>
+        <v>27.676</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>8.093999999999999</v>
+        <v>8.73</v>
       </c>
     </row>
     <row r="9">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>42793754624</v>
+        <v>45003833344</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>13.2125</v>
+        <v>13.893749</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>21.273</v>
+        <v>18.861</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>4.673</v>
+        <v>4.143</v>
       </c>
     </row>
     <row r="10">
@@ -1628,16 +1628,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>339056787456</v>
+        <v>301958594560</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>73.32204</v>
+        <v>65.29944</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>53.196</v>
+        <v>59.64</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>23.762</v>
+        <v>26.641</v>
       </c>
     </row>
     <row r="11">
@@ -1652,16 +1652,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>13474139136</v>
+        <v>13559673856</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>9.800549</v>
+        <v>9.862762999999999</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>8.663</v>
+        <v>8.113</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>1.202</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="12">
@@ -1676,16 +1676,16 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>234540695552</v>
+        <v>285095133184</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>250.24348</v>
+        <v>301.56036</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>153.109</v>
+        <v>192.741</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>21.415</v>
+        <v>26.958</v>
       </c>
     </row>
     <row r="13">
@@ -1700,16 +1700,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>238319943680</v>
+        <v>182832103424</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>24.339075</v>
+        <v>18.65215</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>17.778</v>
+        <v>15.172</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>5.195</v>
+        <v>4.433</v>
       </c>
     </row>
     <row r="15">
@@ -1763,7 +1763,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="35" t="n">
-        <v>0.167</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-03T17:39:05Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -20,11 +20,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.0000"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -126,21 +126,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,9 +150,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -595,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -620,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-02 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-03 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -640,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.92</v>
+        <v>0.952</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -656,7 +657,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -671,10 +672,8 @@
           <t>DCF intrinsic value / share</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B8" s="7" t="n">
+        <v>340.78</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -689,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>137.645</v>
+        <v>137.35</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,10 +702,8 @@
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B10" s="8" t="n">
+        <v>1.481</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -729,8 +726,8 @@
           <t>value_score</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
-        <v>0.873</v>
+      <c r="B13" s="9" t="n">
+        <v>0.874</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -740,7 +737,7 @@
           <t>comps_percentile</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>0.944</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -749,52 +746,67 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>dcf_margin</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Normalized (intrinsic − market) / market, clipped ±50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Honest caveats (read before acting)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
-        </is>
-      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
+          <t>Lite DCF: 5y horizon, 70/30 equity/debt cap structure assumed, FCF growth from 3y trailing trend.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
+          <t>Peer set is FMP's algorithmic /stock-peers — may include weak comps for unusual business models.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
+          <t>Net cash treatment uses cashAndShortTermInvestments (operating cash); excludes LT marketable</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
+          <t xml:space="preserve">  securities, which understates intrinsic for cash-rich companies like AAPL (~$80B in LT inv).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Margin of safety is normalized to 0..1; flip to the DCF tab for the raw % gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>This is a SIGNAL screen, not an investment thesis. Verify with primary filings before acting.</t>
         </is>
@@ -804,6 +816,7 @@
   <mergeCells count="11">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
@@ -812,7 +825,6 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -878,8 +890,8 @@
           <t>Risk-free rate (10y Treasury)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
-        <v>0.04480999946594239</v>
+      <c r="B5" s="10" t="n">
+        <v>0.044849997</v>
       </c>
     </row>
     <row r="6">
@@ -888,7 +900,7 @@
           <t>Equity risk premium (ERP)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -898,8 +910,8 @@
           <t>Beta (levered)</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
-        <v>1.069</v>
+      <c r="B7" s="11" t="n">
+        <v>1.122</v>
       </c>
     </row>
     <row r="8">
@@ -908,7 +920,7 @@
           <t>Credit spread over risk-free</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -918,7 +930,7 @@
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>0.21</v>
       </c>
     </row>
@@ -928,7 +940,7 @@
           <t>Equity weight (cap structure)</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="12" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -938,7 +950,7 @@
           <t>FCF growth (flat, faded avg)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>0.05241951788891955</v>
       </c>
     </row>
@@ -948,7 +960,7 @@
           <t>Terminal growth rate</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -958,7 +970,7 @@
           <t>Latest FCF ($, base year)</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <v>10874360000</v>
       </c>
     </row>
@@ -968,7 +980,7 @@
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="14">
         <f>B5+B7*B6</f>
         <v/>
       </c>
@@ -979,18 +991,18 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="14">
         <f>(B5+B8)*(1-B9)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <f>B10*B15+(1-B10)*B16</f>
         <v/>
       </c>
@@ -1037,23 +1049,23 @@
           <t>Projected FCF</t>
         </is>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="17">
         <f>$B$13*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="17">
         <f>B22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="17">
         <f>C22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="17">
         <f>D22*(1+$B$11)</f>
         <v/>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="17">
         <f>E22*(1+$B$11)</f>
         <v/>
       </c>
@@ -1064,23 +1076,23 @@
           <t>Discount factor</t>
         </is>
       </c>
-      <c r="B23" s="17">
+      <c r="B23" s="18">
         <f>1/(1+$B$17)^1</f>
         <v/>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="18">
         <f>1/(1+$B$17)^2</f>
         <v/>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="18">
         <f>1/(1+$B$17)^3</f>
         <v/>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="18">
         <f>1/(1+$B$17)^4</f>
         <v/>
       </c>
-      <c r="F23" s="17">
+      <c r="F23" s="18">
         <f>1/(1+$B$17)^5</f>
         <v/>
       </c>
@@ -1091,23 +1103,23 @@
           <t>PV of FCF</t>
         </is>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="17">
         <f>B22*B23</f>
         <v/>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="17">
         <f>C22*C23</f>
         <v/>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="17">
         <f>D22*D23</f>
         <v/>
       </c>
-      <c r="E24" s="16">
+      <c r="E24" s="17">
         <f>E22*E23</f>
         <v/>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="17">
         <f>F22*F23</f>
         <v/>
       </c>
@@ -1118,7 +1130,7 @@
           <t>Sum of PV (explicit 5y)</t>
         </is>
       </c>
-      <c r="B26" s="16">
+      <c r="B26" s="17">
         <f>SUM(B24:F24)</f>
         <v/>
       </c>
@@ -1129,7 +1141,7 @@
           <t>Terminal value (Gordon)</t>
         </is>
       </c>
-      <c r="B27" s="16">
+      <c r="B27" s="17">
         <f>F22*(1+B12)/(B17-B12)</f>
         <v/>
       </c>
@@ -1140,18 +1152,18 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="B28" s="16">
+      <c r="B28" s="17">
         <f>B27/(1+B17)^5</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="B29" s="19">
+      <c r="B29" s="20">
         <f>B26+B28</f>
         <v/>
       </c>
@@ -1176,7 +1188,7 @@
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="B32" s="12" t="n">
+      <c r="B32" s="13" t="n">
         <v>8388769792</v>
       </c>
     </row>
@@ -1186,7 +1198,7 @@
           <t>Plus: cash &amp; ST investments</t>
         </is>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B33" s="13" t="n">
         <v>10171567104</v>
       </c>
     </row>
@@ -1196,7 +1208,7 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="B34" s="16">
+      <c r="B34" s="17">
         <f>B29-B32+B33</f>
         <v/>
       </c>
@@ -1207,17 +1219,17 @@
           <t>Diluted shares outstanding</t>
         </is>
       </c>
-      <c r="B35" s="20" t="n">
-        <v>611942072.6651894</v>
+      <c r="B35" s="21" t="n">
+        <v>611942101.7837641</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>Intrinsic per share</t>
         </is>
       </c>
-      <c r="B36" s="21">
+      <c r="B36" s="22">
         <f>B34/B35</f>
         <v/>
       </c>
@@ -1228,17 +1240,17 @@
           <t>Current market price</t>
         </is>
       </c>
-      <c r="B37" s="22" t="n">
-        <v>137.645</v>
+      <c r="B37" s="23" t="n">
+        <v>137.35</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Margin of safety</t>
         </is>
       </c>
-      <c r="B38" s="23">
+      <c r="B38" s="24">
         <f>(B36-B37)/B37</f>
         <v/>
       </c>
@@ -1258,158 +1270,158 @@
       <c r="H41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="inlineStr">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>WACC ↓ / TermG →</t>
         </is>
       </c>
-      <c r="B42" s="25">
+      <c r="B42" s="26">
         <f>$B$12+-0.01</f>
         <v/>
       </c>
-      <c r="C42" s="25">
+      <c r="C42" s="26">
         <f>$B$12+-0.005</f>
         <v/>
       </c>
-      <c r="D42" s="25">
+      <c r="D42" s="26">
         <f>$B$12+0.0</f>
         <v/>
       </c>
-      <c r="E42" s="25">
+      <c r="E42" s="26">
         <f>$B$12+0.005</f>
         <v/>
       </c>
-      <c r="F42" s="25">
+      <c r="F42" s="26">
         <f>$B$12+0.01</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="25">
+      <c r="A43" s="26">
         <f>$B$17+-0.01</f>
         <v/>
       </c>
-      <c r="B43" s="26">
+      <c r="B43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A43-B$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C43" s="26">
+      <c r="C43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A43-C$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D43" s="26">
+      <c r="D43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A43-D$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E43" s="26">
+      <c r="E43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A43-E$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F43" s="26">
+      <c r="F43" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A43)^1+$B$13*(1+$B$11)^2/(1+A43)^2+$B$13*(1+$B$11)^3/(1+A43)^3+$B$13*(1+$B$11)^4/(1+A43)^4+$B$13*(1+$B$11)^5/(1+A43)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A43-F$42))/(1+A43)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="25">
+      <c r="A44" s="26">
         <f>$B$17+-0.005</f>
         <v/>
       </c>
-      <c r="B44" s="26">
+      <c r="B44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A44-B$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C44" s="26">
+      <c r="C44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A44-C$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D44" s="26">
+      <c r="D44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A44-D$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E44" s="26">
+      <c r="E44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A44-E$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F44" s="26">
+      <c r="F44" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A44)^1+$B$13*(1+$B$11)^2/(1+A44)^2+$B$13*(1+$B$11)^3/(1+A44)^3+$B$13*(1+$B$11)^4/(1+A44)^4+$B$13*(1+$B$11)^5/(1+A44)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A44-F$42))/(1+A44)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="25">
+      <c r="A45" s="26">
         <f>$B$17+0.0</f>
         <v/>
       </c>
-      <c r="B45" s="26">
+      <c r="B45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A45-B$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C45" s="26">
+      <c r="C45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A45-C$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D45" s="27">
+      <c r="D45" s="28">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A45-D$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E45" s="26">
+      <c r="E45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A45-E$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F45" s="26">
+      <c r="F45" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A45)^1+$B$13*(1+$B$11)^2/(1+A45)^2+$B$13*(1+$B$11)^3/(1+A45)^3+$B$13*(1+$B$11)^4/(1+A45)^4+$B$13*(1+$B$11)^5/(1+A45)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A45-F$42))/(1+A45)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="25">
+      <c r="A46" s="26">
         <f>$B$17+0.005</f>
         <v/>
       </c>
-      <c r="B46" s="26">
+      <c r="B46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A46-B$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C46" s="26">
+      <c r="C46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A46-C$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D46" s="26">
+      <c r="D46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A46-D$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E46" s="26">
+      <c r="E46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A46-E$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F46" s="26">
+      <c r="F46" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A46)^1+$B$13*(1+$B$11)^2/(1+A46)^2+$B$13*(1+$B$11)^3/(1+A46)^3+$B$13*(1+$B$11)^4/(1+A46)^4+$B$13*(1+$B$11)^5/(1+A46)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A46-F$42))/(1+A46)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="25">
+      <c r="A47" s="26">
         <f>$B$17+0.01</f>
         <v/>
       </c>
-      <c r="B47" s="26">
+      <c r="B47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+B$42)/(A47-B$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="C47" s="26">
+      <c r="C47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+C$42)/(A47-C$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="D47" s="26">
+      <c r="D47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+D$42)/(A47-D$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="E47" s="26">
+      <c r="E47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+E$42)/(A47-E$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
-      <c r="F47" s="26">
+      <c r="F47" s="27">
         <f>($B$13*(1+$B$11)^1/(1+A47)^1+$B$13*(1+$B$11)^2/(1+A47)^2+$B$13*(1+$B$11)^3/(1+A47)^3+$B$13*(1+$B$11)^4/(1+A47)^4+$B$13*(1+$B$11)^5/(1+A47)^5+($B$13*(1+$B$11)^5*(1+F$42)/(A47-F$42))/(1+A47)^5-$B$32+$B$33)/$B$35</f>
         <v/>
       </c>
@@ -1465,59 +1477,59 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C4" s="28" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="D4" s="28" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>P/E (TTM)</t>
         </is>
       </c>
-      <c r="E4" s="28" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="F4" s="28" t="inlineStr">
+      <c r="F4" s="29" t="inlineStr">
         <is>
           <t>EV/Revenue</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>ACN</t>
         </is>
       </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>Accenture plc</t>
         </is>
       </c>
-      <c r="C5" s="30" t="n">
-        <v>84230766592</v>
-      </c>
-      <c r="D5" s="31" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="E5" s="31" t="n">
-        <v>6.19</v>
-      </c>
-      <c r="F5" s="31" t="n">
-        <v>1.09</v>
+      <c r="C5" s="31" t="n">
+        <v>84050247680</v>
+      </c>
+      <c r="D5" s="32" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>1.15</v>
       </c>
     </row>
     <row r="6">
@@ -1531,17 +1543,17 @@
           <t>Adobe Inc.</t>
         </is>
       </c>
-      <c r="C6" s="32" t="n">
-        <v>87986429952</v>
-      </c>
-      <c r="D6" s="33" t="n">
-        <v>12.655775</v>
-      </c>
-      <c r="E6" s="33" t="n">
-        <v>8.769</v>
-      </c>
-      <c r="F6" s="33" t="n">
-        <v>3.386</v>
+      <c r="C6" s="33" t="n">
+        <v>87338696704</v>
+      </c>
+      <c r="D6" s="34" t="n">
+        <v>12.562608</v>
+      </c>
+      <c r="E6" s="34" t="n">
+        <v>9.125999999999999</v>
+      </c>
+      <c r="F6" s="34" t="n">
+        <v>3.524</v>
       </c>
     </row>
     <row r="7">
@@ -1555,17 +1567,17 @@
           <t>Applied Materials, Inc.</t>
         </is>
       </c>
-      <c r="C7" s="32" t="n">
-        <v>465839783936</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>55.299717</v>
-      </c>
-      <c r="E7" s="33" t="n">
-        <v>55.614</v>
-      </c>
-      <c r="F7" s="33" t="n">
-        <v>17.772</v>
+      <c r="C7" s="33" t="n">
+        <v>478789271552</v>
+      </c>
+      <c r="D7" s="34" t="n">
+        <v>56.836945</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>51.517</v>
+      </c>
+      <c r="F7" s="34" t="n">
+        <v>16.463</v>
       </c>
     </row>
     <row r="8">
@@ -1579,17 +1591,17 @@
           <t>Amphenol Corporation</t>
         </is>
       </c>
-      <c r="C8" s="32" t="n">
-        <v>199986921472</v>
-      </c>
-      <c r="D8" s="33" t="n">
-        <v>46.712643</v>
-      </c>
-      <c r="E8" s="33" t="n">
-        <v>27.676</v>
-      </c>
-      <c r="F8" s="33" t="n">
-        <v>8.73</v>
+      <c r="C8" s="33" t="n">
+        <v>202484285440</v>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>47.432274</v>
+      </c>
+      <c r="E8" s="34" t="n">
+        <v>26.528</v>
+      </c>
+      <c r="F8" s="34" t="n">
+        <v>8.368</v>
       </c>
     </row>
     <row r="9">
@@ -1603,17 +1615,17 @@
           <t>Infosys Limited</t>
         </is>
       </c>
-      <c r="C9" s="32" t="n">
-        <v>45003833344</v>
-      </c>
-      <c r="D9" s="33" t="n">
-        <v>13.893749</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <v>18.861</v>
-      </c>
-      <c r="F9" s="33" t="n">
-        <v>4.143</v>
+      <c r="C9" s="33" t="n">
+        <v>45186035712</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="E9" s="34" t="n">
+        <v>19.793</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>4.348</v>
       </c>
     </row>
     <row r="10">
@@ -1627,17 +1639,17 @@
           <t>KLA Corporation</t>
         </is>
       </c>
-      <c r="C10" s="32" t="n">
-        <v>301958594560</v>
-      </c>
-      <c r="D10" s="33" t="n">
-        <v>65.29944</v>
-      </c>
-      <c r="E10" s="33" t="n">
-        <v>59.64</v>
-      </c>
-      <c r="F10" s="33" t="n">
-        <v>26.641</v>
+      <c r="C10" s="33" t="n">
+        <v>307693125632</v>
+      </c>
+      <c r="D10" s="34" t="n">
+        <v>66.72805</v>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>52.798</v>
+      </c>
+      <c r="F10" s="34" t="n">
+        <v>23.585</v>
       </c>
     </row>
     <row r="11">
@@ -1651,17 +1663,17 @@
           <t>Leidos Holdings, Inc.</t>
         </is>
       </c>
-      <c r="C11" s="32" t="n">
-        <v>13559673856</v>
-      </c>
-      <c r="D11" s="33" t="n">
-        <v>9.862762999999999</v>
-      </c>
-      <c r="E11" s="33" t="n">
-        <v>8.113</v>
-      </c>
-      <c r="F11" s="33" t="n">
-        <v>1.125</v>
+      <c r="C11" s="33" t="n">
+        <v>13690489856</v>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>9.957913</v>
+      </c>
+      <c r="E11" s="34" t="n">
+        <v>8.414999999999999</v>
+      </c>
+      <c r="F11" s="34" t="n">
+        <v>1.167</v>
       </c>
     </row>
     <row r="12">
@@ -1675,17 +1687,17 @@
           <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
-      <c r="C12" s="32" t="n">
-        <v>285095133184</v>
-      </c>
-      <c r="D12" s="33" t="n">
-        <v>301.56036</v>
-      </c>
-      <c r="E12" s="33" t="n">
-        <v>192.741</v>
-      </c>
-      <c r="F12" s="33" t="n">
-        <v>26.958</v>
+      <c r="C12" s="33" t="n">
+        <v>283668905984</v>
+      </c>
+      <c r="D12" s="34" t="n">
+        <v>302.6609</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>190.555</v>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>26.652</v>
       </c>
     </row>
     <row r="13">
@@ -1699,17 +1711,17 @@
           <t>QUALCOMM Incorporated</t>
         </is>
       </c>
-      <c r="C13" s="32" t="n">
-        <v>182832103424</v>
-      </c>
-      <c r="D13" s="33" t="n">
-        <v>18.65215</v>
-      </c>
-      <c r="E13" s="33" t="n">
-        <v>15.172</v>
-      </c>
-      <c r="F13" s="33" t="n">
-        <v>4.433</v>
+      <c r="C13" s="33" t="n">
+        <v>185767493632</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>18.931255</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>14.712</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>4.299</v>
       </c>
     </row>
     <row r="15">
@@ -1718,15 +1730,15 @@
           <t>Peer median</t>
         </is>
       </c>
-      <c r="D15" s="34">
+      <c r="D15" s="35">
         <f>MEDIAN(D6:D13)</f>
         <v/>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="35">
         <f>MEDIAN(E6:E13)</f>
         <v/>
       </c>
-      <c r="F15" s="34">
+      <c r="F15" s="35">
         <f>MEDIAN(F6:F13)</f>
         <v/>
       </c>
@@ -1737,15 +1749,15 @@
           <t>Peer mean</t>
         </is>
       </c>
-      <c r="D16" s="34">
+      <c r="D16" s="35">
         <f>AVERAGE(D6:D13)</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="35">
         <f>AVERAGE(E6:E13)</f>
         <v/>
       </c>
-      <c r="F16" s="34">
+      <c r="F16" s="35">
         <f>AVERAGE(F6:F13)</f>
         <v/>
       </c>
@@ -1756,13 +1768,13 @@
           <t>Target percentile vs peers</t>
         </is>
       </c>
-      <c r="D17" s="35" t="n">
+      <c r="D17" s="36" t="n">
         <v>0.167</v>
       </c>
-      <c r="E17" s="35" t="n">
+      <c r="E17" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="35" t="n">
+      <c r="F17" s="36" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-05T17:38:12Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-04 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.044849997</v>
+        <v>0.04485000133514404</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-06T17:38:57Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-05 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-06 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>340.78</v>
+        <v>340.99</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>137.35</v>
+        <v>137.545</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.481</v>
+        <v>1.479</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.874</v>
+        <v>0.873</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04485000133514404</v>
+        <v>0.04480999946594239</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942101.7837641</v>
+        <v>611942072.4272057</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>137.35</v>
+        <v>137.545</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>84050247680</v>
+        <v>84169572352</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>10.96</v>
+        <v>10.98</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>6.48</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>87338696704</v>
+        <v>86992879616</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>12.562608</v>
+        <v>12.512865</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>9.125999999999999</v>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>478789271552</v>
+        <v>470635347968</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>56.836945</v>
+        <v>55.868996</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>51.517</v>
@@ -1592,10 +1592,10 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>202484285440</v>
+        <v>204588007424</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>47.432274</v>
+        <v>47.92507</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>26.528</v>
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>45186035712</v>
+        <v>44639428608</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.95</v>
+        <v>13.781249</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>19.793</v>
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>307693125632</v>
+        <v>303735111680</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>66.72805</v>
+        <v>65.86969000000001</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>52.798</v>
@@ -1664,10 +1664,10 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13690489856</v>
+        <v>13818790912</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>9.957913</v>
+        <v>10.051235</v>
       </c>
       <c r="E11" s="34" t="n">
         <v>8.414999999999999</v>
@@ -1688,10 +1688,10 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>283668905984</v>
+        <v>291024273408</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>302.6609</v>
+        <v>310.5087</v>
       </c>
       <c r="E12" s="34" t="n">
         <v>190.555</v>
@@ -1712,10 +1712,10 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>185767493632</v>
+        <v>196191551488</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.931255</v>
+        <v>19.993555</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>14.712</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-16T17:40:03Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-06 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-16 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.952</v>
+        <v>0.95</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>340.99</v>
+        <v>336.25</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>137.545</v>
+        <v>143.3</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.479</v>
+        <v>1.346</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.873</v>
+        <v>0.861</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04480999946594239</v>
+        <v>0.04572999954223633</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942072.4272057</v>
+        <v>611942114.1660851</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>137.545</v>
+        <v>143.3</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>84169572352</v>
+        <v>87691304960</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>10.98</v>
+        <v>11.45</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.48</v>
+        <v>6.46</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>1.15</v>
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>86992879616</v>
+        <v>92685074432</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>12.512865</v>
+        <v>13.346881</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.125999999999999</v>
+        <v>9.324</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.524</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>470635347968</v>
+        <v>445693067264</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>55.868996</v>
+        <v>52.958015</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>51.517</v>
+        <v>49.496</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>16.463</v>
+        <v>15.817</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>204588007424</v>
+        <v>188877897728</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>47.92507</v>
+        <v>43.9914</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>26.528</v>
+        <v>25.391</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>8.368</v>
+        <v>8.01</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>44639428608</v>
+        <v>46339981312</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.781249</v>
+        <v>14.30625</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.793</v>
+        <v>19.573</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.348</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>303735111680</v>
+        <v>286557569024</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>65.86969000000001</v>
+        <v>62.321022</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>52.798</v>
+        <v>50.331</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>23.585</v>
+        <v>22.483</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13818790912</v>
+        <v>13738288128</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>10.051235</v>
+        <v>9.992680999999999</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.414999999999999</v>
+        <v>8.382</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.167</v>
+        <v>1.163</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>291024273408</v>
+        <v>286280974336</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>310.5087</v>
+        <v>310.854</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>190.555</v>
+        <v>193.829</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>26.652</v>
+        <v>27.11</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>196191551488</v>
+        <v>180265615360</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>19.993555</v>
+        <v>18.37057</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.712</v>
+        <v>14.852</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.299</v>
+        <v>4.34</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-17T17:40:23Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-16 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-17 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.95</v>
+        <v>0.928</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>336.25</v>
+        <v>337.42</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>143.3</v>
+        <v>143.205</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.346</v>
+        <v>1.356</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.944</v>
+        <v>0.889</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04572999954223633</v>
+        <v>0.04550000190734863</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942114.1660851</v>
+        <v>611942085.374114</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>143.3</v>
+        <v>143.205</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>87691304960</v>
+        <v>87633166336</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.45</v>
+        <v>11.44</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.46</v>
+        <v>6.82</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.15</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>92685074432</v>
+        <v>95157526528</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.346881</v>
+        <v>13.695081</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.324</v>
+        <v>9.763</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.6</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>445693067264</v>
+        <v>429480443904</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>52.958015</v>
+        <v>50.744373</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>49.496</v>
+        <v>47.912</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>15.817</v>
+        <v>15.311</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>188877897728</v>
+        <v>188145909760</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>43.9914</v>
+        <v>43.94684</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>25.391</v>
+        <v>24.804</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>8.01</v>
+        <v>7.824</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>46339981312</v>
+        <v>46216491008</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.30625</v>
+        <v>14.268126</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.573</v>
+        <v>20.469</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.3</v>
+        <v>4.496</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>286557569024</v>
+        <v>280744656896</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>62.321022</v>
+        <v>60.883854</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>50.331</v>
+        <v>49.185</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>22.483</v>
+        <v>21.971</v>
       </c>
     </row>
     <row r="11">
@@ -1664,13 +1664,13 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13738288128</v>
+        <v>13382943744</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>9.992680999999999</v>
+        <v>9.734218</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.382</v>
+        <v>8.385999999999999</v>
       </c>
       <c r="F11" s="34" t="n">
         <v>1.163</v>
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>286280974336</v>
+        <v>294875136000</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>310.854</v>
+        <v>320.18585</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>193.829</v>
+        <v>193.813</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>27.11</v>
+        <v>27.108</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>180265615360</v>
+        <v>179901988864</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.37057</v>
+        <v>18.353226</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.852</v>
+        <v>14.254</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.34</v>
+        <v>4.165</v>
       </c>
     </row>
     <row r="15">
@@ -1775,7 +1775,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="36" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-18T17:38:27Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-17 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-18 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>337.42</v>
+        <v>337.89</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>143.205</v>
+        <v>143.57</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.356</v>
+        <v>1.353</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04550000190734863</v>
+        <v>0.04540999889373779</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942085.374114</v>
+        <v>611942114.7036289</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>143.205</v>
+        <v>143.57</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>87633166336</v>
+        <v>87856529408</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.44</v>
+        <v>11.47</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.82</v>
+        <v>6.78</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>95157526528</v>
+        <v>94306877440</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.695081</v>
+        <v>13.564895</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.763</v>
+        <v>9.843</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.77</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>429480443904</v>
+        <v>420528521216</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>50.744373</v>
+        <v>49.733334</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>47.912</v>
+        <v>45.235</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>15.311</v>
+        <v>14.455</v>
       </c>
     </row>
     <row r="8">
@@ -1588,20 +1588,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Amphenol Corporation</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>188145909760</v>
+        <v>186011451392</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>43.94684</v>
+        <v>43.448277</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.804</v>
+        <v>24.512</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.824</v>
+        <v>7.732</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>46216491008</v>
+        <v>46522183680</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.268126</v>
+        <v>14.362499</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>20.469</v>
+        <v>20.396</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.496</v>
+        <v>4.48</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>280744656896</v>
+        <v>277910061056</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>60.883854</v>
+        <v>62.026237</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>49.185</v>
+        <v>47.707</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>21.971</v>
+        <v>21.311</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13382943744</v>
+        <v>13393636352</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>9.734218</v>
+        <v>9.750916</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.385999999999999</v>
+        <v>8.291</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.163</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>294875136000</v>
+        <v>292324179968</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>320.18585</v>
+        <v>311.89566</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>193.813</v>
+        <v>196.389</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>27.108</v>
+        <v>27.468</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>179901988864</v>
+        <v>181056110592</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.353226</v>
+        <v>18.49085</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.254</v>
+        <v>14.349</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.165</v>
+        <v>4.193</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-19T17:38:45Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-18 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-19 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>Amphenol Corporation</t>
         </is>
       </c>
       <c r="C8" s="33" t="n">
@@ -1643,7 +1643,7 @@
         <v>277910061056</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>62.026237</v>
+        <v>60.269123</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>47.707</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-20T17:40:08Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-19 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-20 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.928</v>
+        <v>0.927</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>337.89</v>
+        <v>334.68</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>143.57</v>
+        <v>144.96</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.353</v>
+        <v>1.309</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.861</v>
+        <v>0.858</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04540999889373779</v>
+        <v>0.04604000091552735</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942114.7036289</v>
+        <v>611942117.4392936</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>143.57</v>
+        <v>144.96</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>87856529408</v>
+        <v>88707129344</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.47</v>
+        <v>11.58</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>6.78</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>94306877440</v>
+        <v>93472120832</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.564895</v>
+        <v>13.444825</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>9.843</v>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>420528521216</v>
+        <v>421798903808</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>49.733334</v>
+        <v>49.88357</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>45.235</v>
@@ -1591,11 +1591,9 @@
           <t>Amphenol Corporation</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n">
-        <v>186011451392</v>
-      </c>
+      <c r="C8" s="33" t="n"/>
       <c r="D8" s="34" t="n">
-        <v>43.448277</v>
+        <v>43.5273</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>24.512</v>
@@ -1616,10 +1614,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>46522183680</v>
+        <v>46501937152</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.362499</v>
+        <v>14.35625</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>20.396</v>
@@ -1640,10 +1638,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>277910061056</v>
+        <v>274043469824</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>60.269123</v>
+        <v>59.43059</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>47.707</v>
@@ -1664,10 +1662,10 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13393636352</v>
+        <v>13478541312</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>9.750916</v>
+        <v>9.812728999999999</v>
       </c>
       <c r="E11" s="34" t="n">
         <v>8.291</v>
@@ -1688,10 +1686,10 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>292324179968</v>
+        <v>294227247104</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>311.89566</v>
+        <v>313.92612</v>
       </c>
       <c r="E12" s="34" t="n">
         <v>196.389</v>
@@ -1712,10 +1710,10 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>181056110592</v>
+        <v>181182595072</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.49085</v>
+        <v>18.503767</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>14.349</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-07-21T17:40:25Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-20 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-21 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.927</v>
+        <v>0.929</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>334.68</v>
+        <v>333.58</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>144.96</v>
+        <v>140.5301</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.309</v>
+        <v>1.374</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.858</v>
+        <v>0.867</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04604000091552735</v>
+        <v>0.04625999927520752</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942117.4392936</v>
+        <v>611942081.1342196</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>144.96</v>
+        <v>140.5301</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>88707129344</v>
+        <v>85996281856</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.58</v>
+        <v>11.22</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.78</v>
+        <v>6.83</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>93472120832</v>
+        <v>89890652160</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>13.444825</v>
+        <v>12.929674</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.843</v>
+        <v>9.74</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.8</v>
+        <v>3.761</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>421798903808</v>
+        <v>451758948352</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>49.88357</v>
+        <v>53.577682</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>45.235</v>
+        <v>44.896</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>14.455</v>
+        <v>14.347</v>
       </c>
     </row>
     <row r="8">
@@ -1591,15 +1591,17 @@
           <t>Amphenol Corporation</t>
         </is>
       </c>
-      <c r="C8" s="33" t="n"/>
+      <c r="C8" s="33" t="n">
+        <v>193811136512</v>
+      </c>
       <c r="D8" s="34" t="n">
-        <v>43.5273</v>
+        <v>45.27011</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.512</v>
+        <v>24.408</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.732</v>
+        <v>7.699</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>46501937152</v>
+        <v>45408727040</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.35625</v>
+        <v>14.01875</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>20.396</v>
+        <v>20.067</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.48</v>
+        <v>4.408</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>274043469824</v>
+        <v>285414588416</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>59.43059</v>
+        <v>61.8966</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>47.707</v>
+        <v>46.557</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>21.311</v>
+        <v>20.797</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13478541312</v>
+        <v>13170996224</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>9.812728999999999</v>
+        <v>9.580054000000001</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.291</v>
+        <v>8.319000000000001</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.15</v>
+        <v>1.154</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>294227247104</v>
+        <v>274695733248</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>313.92612</v>
+        <v>293.08694</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>196.389</v>
+        <v>190.884</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>27.468</v>
+        <v>26.698</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>181182595072</v>
+        <v>182626582528</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.503767</v>
+        <v>18.631184</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.349</v>
+        <v>14.231</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.193</v>
+        <v>4.158</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-22T17:40:11Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-21 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-22 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>333.58</v>
+        <v>332.18</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>140.5301</v>
+        <v>139.75</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.374</v>
+        <v>1.377</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.867</v>
+        <v>0.869</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04625999927520752</v>
+        <v>0.04654000282287598</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942081.1342196</v>
+        <v>611942106.9051878</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>140.5301</v>
+        <v>139.75</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>85996281856</v>
+        <v>85518909440</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.22</v>
+        <v>11.16</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.83</v>
+        <v>6.65</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.21</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>89890652160</v>
+        <v>87748124672</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>12.929674</v>
+        <v>12.621498</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.74</v>
+        <v>9.43</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.761</v>
+        <v>3.641</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>451758948352</v>
+        <v>444287811584</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>53.577682</v>
+        <v>52.741287</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>44.896</v>
+        <v>48.222</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>14.347</v>
+        <v>15.41</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>193811136512</v>
+        <v>193515896832</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>45.27011</v>
+        <v>45.071632</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.408</v>
+        <v>25.507</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.699</v>
+        <v>8.045999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>45408727040</v>
+        <v>44072583168</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.01875</v>
+        <v>13.60625</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>20.067</v>
+        <v>19.793</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.408</v>
+        <v>4.348</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>285414588416</v>
+        <v>282455867392</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>61.8966</v>
+        <v>61.428978</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>46.557</v>
+        <v>48.781</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>20.797</v>
+        <v>21.79</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13170996224</v>
+        <v>13508101120</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>9.580054000000001</v>
+        <v>9.825252000000001</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.319000000000001</v>
+        <v>8.209</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.154</v>
+        <v>1.139</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>274695733248</v>
+        <v>274104877056</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>293.08694</v>
+        <v>289.93536</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>190.884</v>
+        <v>187.308</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>26.698</v>
+        <v>26.198</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>182626582528</v>
+        <v>186210172928</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.631184</v>
+        <v>18.996773</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.231</v>
+        <v>14.489</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.158</v>
+        <v>4.234</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-24T17:40:34Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-22 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-24 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.929</v>
+        <v>0.949</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>332.18</v>
+        <v>331.24</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>139.75</v>
+        <v>145.645</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.377</v>
+        <v>1.274</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.869</v>
+        <v>0.856</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.889</v>
+        <v>0.944</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04654000282287598</v>
+        <v>0.04672999858856201</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942106.9051878</v>
+        <v>611942090.6450616</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>139.75</v>
+        <v>145.645</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>85518909440</v>
+        <v>89126305792</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.16</v>
+        <v>11.64</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.65</v>
+        <v>6.55</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>87748124672</v>
+        <v>88881037312</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>12.621498</v>
+        <v>12.791768</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.43</v>
+        <v>8.818</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.641</v>
+        <v>3.405</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>444287811584</v>
+        <v>436185432064</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>52.741287</v>
+        <v>51.633457</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>48.222</v>
+        <v>48.072</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>15.41</v>
+        <v>15.362</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>193515896832</v>
+        <v>191036964864</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>45.071632</v>
+        <v>44.622128</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>25.507</v>
+        <v>25.45</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>8.045999999999999</v>
+        <v>8.028</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>44072583168</v>
+        <v>44490604544</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.60625</v>
+        <v>13.561728</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.793</v>
+        <v>19.372</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.348</v>
+        <v>4.255</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>282455867392</v>
+        <v>280496472064</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>61.428978</v>
+        <v>61.00284</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>48.781</v>
+        <v>49.042</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>21.79</v>
+        <v>21.907</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>13508101120</v>
+        <v>14246461440</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>9.825252000000001</v>
+        <v>10.362306</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.209</v>
+        <v>8.492000000000001</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.139</v>
+        <v>1.178</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>274104877056</v>
+        <v>265861136384</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>289.93536</v>
+        <v>286.1491</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>187.308</v>
+        <v>178.232</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>26.198</v>
+        <v>24.929</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>186210172928</v>
+        <v>178210324480</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.996773</v>
+        <v>18.161116</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.489</v>
+        <v>14.295</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.234</v>
+        <v>4.177</v>
       </c>
     </row>
     <row r="15">
@@ -1775,7 +1775,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="36" t="n">
-        <v>0.167</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-25T17:39:11Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-24 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-25 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.949</v>
+        <v>0.926</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>331.24</v>
+        <v>330.95</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>145.645</v>
+        <v>146.99</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.274</v>
+        <v>1.252</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.856</v>
+        <v>0.853</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.944</v>
+        <v>0.889</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04672999858856201</v>
+        <v>0.04678999900817871</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942090.6450616</v>
+        <v>611942121.3415878</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>145.645</v>
+        <v>146.99</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>89126305792</v>
+        <v>89949372416</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.64</v>
+        <v>11.74</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.55</v>
+        <v>6.94</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.16</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>88881037312</v>
+        <v>89481224192</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>12.791768</v>
+        <v>12.870784</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>8.818</v>
+        <v>9.347</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.405</v>
+        <v>3.609</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>436185432064</v>
+        <v>425760751616</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>51.633457</v>
+        <v>50.49435</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>48.072</v>
+        <v>45.799</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>15.362</v>
+        <v>14.636</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>191036964864</v>
+        <v>187819900928</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>44.622128</v>
+        <v>43.87069</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>25.45</v>
+        <v>24.733</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>8.028</v>
+        <v>7.802</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>44490604544</v>
+        <v>44996870144</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.561728</v>
+        <v>13.716049</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.372</v>
+        <v>19.598</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.255</v>
+        <v>4.327</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>280496472064</v>
+        <v>274997051392</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>61.00284</v>
+        <v>59.46893</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>49.042</v>
+        <v>47.209</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>21.907</v>
+        <v>21.088</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14246461440</v>
+        <v>14105581568</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>10.362306</v>
+        <v>10.259835</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.492000000000001</v>
+        <v>8.587</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.178</v>
+        <v>1.191</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>265861136384</v>
+        <v>263888863232</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>286.1491</v>
+        <v>276.74362</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>178.232</v>
+        <v>177.221</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>24.929</v>
+        <v>24.787</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>178210324480</v>
+        <v>175986376704</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.161116</v>
+        <v>17.953764</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.295</v>
+        <v>13.959</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.177</v>
+        <v>4.079</v>
       </c>
     </row>
     <row r="15">
@@ -1775,7 +1775,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="36" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-18T17:44:15Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-25 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-18 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.926</v>
+        <v>0.914</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>330.95</v>
+        <v>338.31</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>146.99</v>
+        <v>176.22</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.252</v>
+        <v>0.92</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.853</v>
+        <v>0.791</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04678999900817871</v>
+        <v>0.04711999893188477</v>
       </c>
     </row>
     <row r="6">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1.122</v>
+        <v>1.074</v>
       </c>
     </row>
     <row r="8">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942121.3415878</v>
+        <v>611942074.5885825</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>146.99</v>
+        <v>176.22</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>89949372416</v>
+        <v>107836432384</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.74</v>
+        <v>14.06</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>6.94</v>
+        <v>8.02</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.23</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>89481224192</v>
+        <v>105923813376</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>12.870784</v>
+        <v>15.244566</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>9.347</v>
+        <v>10.529</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.609</v>
+        <v>4.065</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>425760751616</v>
+        <v>401346494464</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>50.49435</v>
+        <v>43.502583</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>45.799</v>
+        <v>41.59</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>14.636</v>
+        <v>13.696</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>187819900928</v>
+        <v>195908730880</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>43.87069</v>
+        <v>39.7225</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.733</v>
+        <v>23.691</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.802</v>
+        <v>7.728</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>44996870144</v>
+        <v>48358473728</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.716049</v>
+        <v>14.74074</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.598</v>
+        <v>20.519</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.327</v>
+        <v>4.531</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>274997051392</v>
+        <v>253378609152</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>59.46893</v>
+        <v>52.986336</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>47.209</v>
+        <v>44.607</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>21.088</v>
+        <v>19.889</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>14105581568</v>
+        <v>18237782016</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>10.259835</v>
+        <v>13.569561</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>8.587</v>
+        <v>9.964</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.191</v>
+        <v>1.346</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>263888863232</v>
+        <v>304810000384</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>276.74362</v>
+        <v>322.4138</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>177.221</v>
+        <v>205.772</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>24.787</v>
+        <v>28.781</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>175986376704</v>
+        <v>166876921856</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>17.953764</v>
+        <v>18.138699</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>13.959</v>
+        <v>14.776</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.079</v>
+        <v>4.023</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-19T17:43:20Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-18 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-19 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.914</v>
+        <v>0.91</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>338.31</v>
+        <v>340.28</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>176.22</v>
+        <v>184.085</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.92</v>
+        <v>0.848</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.791</v>
+        <v>0.774</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04711999893188477</v>
+        <v>0.04674000263214111</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942074.5885825</v>
+        <v>611942110.7423201</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>176.22</v>
+        <v>184.085</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>107836432384</v>
+        <v>112649363456</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.06</v>
+        <v>14.7</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.02</v>
+        <v>8.16</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.42</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>105923813376</v>
+        <v>108167700480</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>15.244566</v>
+        <v>15.576417</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.529</v>
+        <v>10.9</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>4.065</v>
+        <v>4.209</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>401346494464</v>
+        <v>392323137536</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>43.502583</v>
+        <v>42.708298</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>41.59</v>
+        <v>39.95</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>13.696</v>
+        <v>13.156</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>195908730880</v>
+        <v>193239334912</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>39.7225</v>
+        <v>39.08354</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>23.691</v>
+        <v>22.219</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.728</v>
+        <v>7.248</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>48358473728</v>
+        <v>49188753408</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.74074</v>
+        <v>14.993828</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>20.519</v>
+        <v>20.899</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.531</v>
+        <v>4.614</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>253378609152</v>
+        <v>244781547520</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>52.986336</v>
+        <v>51.188526</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>44.607</v>
+        <v>42.24</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>19.889</v>
+        <v>18.834</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>18237782016</v>
+        <v>18465552384</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>13.569561</v>
+        <v>13.75187</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.964</v>
+        <v>10.028</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.346</v>
+        <v>1.355</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>304810000384</v>
+        <v>291721117696</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>322.4138</v>
+        <v>308.56897</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>205.772</v>
+        <v>204.882</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>28.781</v>
+        <v>28.656</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>166876921856</v>
+        <v>170442457088</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.138699</v>
+        <v>18.76185</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.776</v>
+        <v>14.601</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.023</v>
+        <v>3.976</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-21T17:42:21Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-19 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-21 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>340.28</v>
+        <v>337.18</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>184.085</v>
+        <v>185.32</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.848</v>
+        <v>0.819</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.774</v>
+        <v>0.772</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04674000263214111</v>
+        <v>0.04734000205993652</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942110.7423201</v>
+        <v>611942090.5676668</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>184.085</v>
+        <v>185.32</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>112649363456</v>
+        <v>113405108224</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.7</v>
+        <v>14.81</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.16</v>
+        <v>8.56</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.45</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>108167700480</v>
+        <v>109138001920</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>15.576417</v>
+        <v>15.707151</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.9</v>
+        <v>11.271</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>4.209</v>
+        <v>4.352</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>392323137536</v>
+        <v>388246142976</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>42.708298</v>
+        <v>42.118866</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>39.95</v>
+        <v>38.533</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>13.156</v>
+        <v>12.689</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>193239334912</v>
+        <v>193461256192</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>39.08354</v>
+        <v>39.22625</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>22.219</v>
+        <v>21.377</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.248</v>
+        <v>6.973</v>
       </c>
     </row>
     <row r="9">
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>49188753408</v>
+        <v>48621731840</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.993828</v>
+        <v>14.820988</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>20.899</v>
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>244781547520</v>
+        <v>240110632960</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>51.188526</v>
+        <v>50.211746</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>42.24</v>
+        <v>40.313</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>18.834</v>
+        <v>17.974</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>18465552384</v>
+        <v>17770323968</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>13.75187</v>
+        <v>13.209421</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>10.028</v>
+        <v>9.917</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.355</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>291721117696</v>
+        <v>292128587776</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>308.56897</v>
+        <v>311.68695</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>204.882</v>
+        <v>191.379</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>28.656</v>
+        <v>26.768</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>170442457088</v>
+        <v>168720072704</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.76185</v>
+        <v>18.381006</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.601</v>
+        <v>14.65</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>3.976</v>
+        <v>3.989</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-08-22T17:40:54Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-22 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.91</v>
+        <v>0.888</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>337.18</v>
+        <v>336.98</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>185.32</v>
+        <v>185.28</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.889</v>
+        <v>0.833</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04734000205993652</v>
+        <v>0.0473799991607666</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942090.5676668</v>
+        <v>611942090.5008636</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>185.32</v>
+        <v>185.28</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>113405108224</v>
+        <v>113380630528</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.81</v>
+        <v>14.8</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.56</v>
+        <v>8.75</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>109138001920</v>
+        <v>109431742464</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>15.707151</v>
+        <v>15.749428</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>11.271</v>
+        <v>11.397</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>4.352</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>388246142976</v>
+        <v>390882099200</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>42.118866</v>
+        <v>42.55143</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>38.533</v>
+        <v>38.288</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>12.689</v>
+        <v>12.609</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>193461256192</v>
+        <v>193590722560</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>39.22625</v>
+        <v>39.2525</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>21.377</v>
+        <v>21.885</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>6.973</v>
+        <v>7.139</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>48621731840</v>
+        <v>48358473728</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.820988</v>
+        <v>14.560975</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>20.899</v>
+        <v>21.098</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.614</v>
+        <v>4.658</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>240110632960</v>
+        <v>240391553024</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>50.211746</v>
+        <v>50.270493</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>40.313</v>
+        <v>39.909</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>17.974</v>
+        <v>17.795</v>
       </c>
     </row>
     <row r="11">
@@ -1664,13 +1664,13 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>17770323968</v>
+        <v>17743343616</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>13.209421</v>
+        <v>13.214019</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.917</v>
+        <v>9.917999999999999</v>
       </c>
       <c r="F11" s="34" t="n">
         <v>1.34</v>
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>292128587776</v>
+        <v>291664035840</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>311.68695</v>
+        <v>311.1913</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>191.379</v>
+        <v>195.944</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>26.768</v>
+        <v>27.406</v>
       </c>
     </row>
     <row r="13">
@@ -1712,10 +1712,10 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>168720072704</v>
+        <v>168825110528</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.381006</v>
+        <v>18.392448</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>14.65</v>
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D17" s="36" t="n">
-        <v>0.167</v>
+        <v>0.333</v>
       </c>
       <c r="E17" s="36" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-09-10T17:43:57Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-22 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-10 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.888</v>
+        <v>0.891</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>336.98</v>
+        <v>324.63</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>185.28</v>
+        <v>177.73</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.819</v>
+        <v>0.827</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.772</v>
+        <v>0.788</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.0473799991607666</v>
+        <v>0.0492199993133545</v>
       </c>
     </row>
     <row r="6">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1.074</v>
+        <v>1.092</v>
       </c>
     </row>
     <row r="8">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942090.5008636</v>
+        <v>611942077.3532888</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>185.28</v>
+        <v>177.73</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>113380630528</v>
+        <v>108760465408</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.8</v>
+        <v>14.2</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.75</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.55</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>109431742464</v>
+        <v>99150413824</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>15.749428</v>
+        <v>14.269737</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>11.397</v>
+        <v>10.562</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>4.4</v>
+        <v>4.078</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>390882099200</v>
+        <v>363233509376</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>42.55143</v>
+        <v>39.525475</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>38.288</v>
+        <v>36.454</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>12.609</v>
+        <v>12.005</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>193590722560</v>
+        <v>197240356864</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>39.2525</v>
+        <v>39.9925</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>21.885</v>
+        <v>22.624</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.139</v>
+        <v>7.38</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>48358473728</v>
+        <v>43945750528</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.560975</v>
+        <v>13.395062</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>21.098</v>
+        <v>19.272</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.658</v>
+        <v>4.255</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>240391553024</v>
+        <v>232473870336</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>50.270493</v>
+        <v>50.121124</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>39.909</v>
+        <v>39.676</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>17.795</v>
+        <v>17.691</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>17743343616</v>
+        <v>16231161856</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>13.214019</v>
+        <v>12.076564</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.917999999999999</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.34</v>
+        <v>1.245</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>291664035840</v>
+        <v>277165178880</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>311.1913</v>
+        <v>298.3158</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>195.944</v>
+        <v>146.806</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>27.406</v>
+        <v>23.798</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>168825110528</v>
+        <v>192460554240</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>18.392448</v>
+        <v>20.593863</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>14.65</v>
+        <v>16.02</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>3.989</v>
+        <v>4.362</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-09-11T17:44:36Z
</commit_message>
<xml_diff>
--- a/app/reports/ACN_research.xlsx
+++ b/app/reports/ACN_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-10 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-11 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.891</v>
+        <v>0.867</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>324.63</v>
+        <v>323.45</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>177.73</v>
+        <v>181.3001</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.827</v>
+        <v>0.784</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.788</v>
+        <v>0.78</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.833</v>
+        <v>0.778</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.0492199993133545</v>
+        <v>0.04947000026702881</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>611942077.3532888</v>
+        <v>611942062.4699049</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>177.73</v>
+        <v>181.3001</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>108760465408</v>
+        <v>110945157120</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>14.2</v>
+        <v>14.48</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.47</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>99150413824</v>
+        <v>100933197824</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>14.269737</v>
+        <v>14.169642</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.562</v>
+        <v>10.316</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>4.078</v>
+        <v>3.983</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>363233509376</v>
+        <v>365896040448</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>39.525475</v>
+        <v>39.815197</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>36.454</v>
+        <v>35.294</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>12.005</v>
+        <v>11.623</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>197240356864</v>
+        <v>206216478720</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>39.9925</v>
+        <v>41.8125</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>22.624</v>
+        <v>22.34</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>7.38</v>
+        <v>7.287</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>43945750528</v>
+        <v>44411535360</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>13.395062</v>
+        <v>13.537037</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>19.272</v>
+        <v>19.236</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>4.255</v>
+        <v>4.247</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>232473870336</v>
+        <v>237268910080</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>50.121124</v>
+        <v>49.48229</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>39.676</v>
+        <v>38.44</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>17.691</v>
+        <v>17.139</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>16231161856</v>
+        <v>16055473152</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>12.076564</v>
+        <v>11.945846</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>9.220000000000001</v>
+        <v>9.295</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>1.245</v>
+        <v>1.256</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>277165178880</v>
+        <v>268130926592</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>298.3158</v>
+        <v>286.0826</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>146.806</v>
+        <v>148.294</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>23.798</v>
+        <v>24.04</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>192460554240</v>
+        <v>197847531520</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>20.593863</v>
+        <v>21.146118</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>16.02</v>
+        <v>16.062</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>4.362</v>
+        <v>4.373</v>
       </c>
     </row>
     <row r="15">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="D17" s="36" t="n">
-        <v>0.333</v>
+        <v>0.5</v>
       </c>
       <c r="E17" s="36" t="n">
         <v>0</v>

</xml_diff>